<commit_message>
finish CG begin test GA
</commit_message>
<xml_diff>
--- a/candidate_points.xlsx
+++ b/candidate_points.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="8055"/>
+    <workbookView windowWidth="21094" windowHeight="9805"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1033,9 +1033,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.1" outlineLevelCol="4"/>
   <cols>
-    <col min="3" max="3" width="16.2654867256637" customWidth="1"/>
+    <col min="3" max="3" width="16.2612612612613" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1070,7 +1070,7 @@
         <v>31.2809145</v>
       </c>
       <c r="E2">
-        <v>500</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1087,7 +1087,7 @@
         <v>31.2809145</v>
       </c>
       <c r="E3">
-        <v>501</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1104,7 +1104,7 @@
         <v>31.2809145</v>
       </c>
       <c r="E4">
-        <v>502</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1121,7 +1121,7 @@
         <v>31.29804887</v>
       </c>
       <c r="E5">
-        <v>503</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1138,7 +1138,7 @@
         <v>31.27624149</v>
       </c>
       <c r="E6">
-        <v>504</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1155,7 +1155,7 @@
         <v>31.27468382</v>
       </c>
       <c r="E7">
-        <v>505</v>
+        <v>205</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1172,7 +1172,7 @@
         <v>31.27468382</v>
       </c>
       <c r="E8">
-        <v>506</v>
+        <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1189,7 +1189,7 @@
         <v>31.27468382</v>
       </c>
       <c r="E9">
-        <v>507</v>
+        <v>207</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1206,7 +1206,7 @@
         <v>31.27312615</v>
       </c>
       <c r="E10">
-        <v>508</v>
+        <v>208</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1223,7 +1223,7 @@
         <v>31.27624149</v>
       </c>
       <c r="E11">
-        <v>509</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1240,7 +1240,7 @@
         <v>31.27468382</v>
       </c>
       <c r="E12">
-        <v>510</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1257,7 +1257,7 @@
         <v>31.27468382</v>
       </c>
       <c r="E13">
-        <v>511</v>
+        <v>211</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1274,7 +1274,7 @@
         <v>31.26845314</v>
       </c>
       <c r="E14">
-        <v>512</v>
+        <v>212</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1291,7 +1291,7 @@
         <v>31.26845314</v>
       </c>
       <c r="E15">
-        <v>513</v>
+        <v>213</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1308,7 +1308,7 @@
         <v>31.27001081</v>
       </c>
       <c r="E16">
-        <v>514</v>
+        <v>214</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1325,7 +1325,7 @@
         <v>31.27156848</v>
       </c>
       <c r="E17">
-        <v>515</v>
+        <v>215</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1342,7 +1342,7 @@
         <v>31.28870285</v>
       </c>
       <c r="E18">
-        <v>516</v>
+        <v>216</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1359,7 +1359,7 @@
         <v>31.28870285</v>
       </c>
       <c r="E19">
-        <v>517</v>
+        <v>217</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1376,7 +1376,7 @@
         <v>31.28714518</v>
       </c>
       <c r="E20">
-        <v>518</v>
+        <v>218</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1393,7 +1393,7 @@
         <v>31.28402984</v>
       </c>
       <c r="E21">
-        <v>519</v>
+        <v>219</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1410,7 +1410,7 @@
         <v>31.2653378</v>
       </c>
       <c r="E22">
-        <v>520</v>
+        <v>220</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1427,7 +1427,7 @@
         <v>31.2653378</v>
       </c>
       <c r="E23">
-        <v>521</v>
+        <v>221</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1444,7 +1444,7 @@
         <v>31.2653378</v>
       </c>
       <c r="E24">
-        <v>522</v>
+        <v>222</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1461,7 +1461,7 @@
         <v>31.2653378</v>
       </c>
       <c r="E25">
-        <v>523</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>